<commit_message>
Docs : prompts ajustés aux avatars retenus (Lydia cheveux mi-longs, Marc sourire)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142Mr13BCgQRDKKKVw1X1e6
</commit_message>
<xml_diff>
--- a/docs/prompts-lydia-marc-othmane.xlsx
+++ b/docs/prompts-lydia-marc-othmane.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -719,7 +719,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Voici mon personnage de référence (image jointe). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage (buste centré, tête au même endroit), même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche est fermée, détendue et neutre (pas de sourire, pas de dents visibles), les yeux ouverts (blanc de l'œil et pupille visibles) regardant droit vers la caméra, sourcils au repos, expression calme et neutre. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici mon personnage de référence (image jointe). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage (buste centré, tête au même endroit), même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche est fermée, détendue et neutre (pas de sourire, pas de dents visibles), les yeux ouverts (blanc de l'œil et pupille visibles) regardant droit vers la caméra, sourcils au repos, expression calme et neutre. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres fermées et légèrement pressées l'une contre l'autre, comme au début du son « M » ou « P », un peu plus fermes que dans la base ; yeux, sourcils et tout le reste inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres fermées et légèrement pressées l'une contre l'autre, comme au début du son « M » ou « P », un peu plus fermes que dans la base ; yeux, sourcils et tout le reste inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres légèrement entrouvertes laissant voir les dents du haut et du bas serrées, ouverture très faible, pas de langue ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres légèrement entrouvertes laissant voir les dents du haut et du bas serrées, ouverture très faible, pas de langue ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -839,7 +839,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : ouverte à moitié, forme légèrement ovale, dents du haut visibles, mâchoire un peu abaissée ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : ouverte à moitié, forme légèrement ovale, dents du haut visibles, mâchoire un peu abaissée ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : grande ouverte, mâchoire nettement abaissée, forme ovale verticale, dents du haut visibles, intérieur visible ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : grande ouverte, mâchoire nettement abaissée, forme ovale verticale, dents du haut visibles, intérieur visible ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres arrondies formant un « O » ouvert de taille moyenne, intérieur sombre visible ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres arrondies formant un « O » ouvert de taille moyenne, intérieur sombre visible ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres pincées et projetées vers l'avant en un petit cercle serré, comme pour le son « OU » ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres pincées et projetées vers l'avant en un petit cercle serré, comme pour le son « OU » ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvre inférieure repliée vers l'intérieur, touchant les dents du haut visibles, lèvre supérieure normale, ouverture faible ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvre inférieure repliée vers l'intérieur, touchant les dents du haut visibles, lèvre supérieure normale, ouverture faible ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : ouverte moyennement, pointe de la langue relevée et visible touchant l'arrière des dents du haut ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : ouverte moyennement, pointe de la langue relevée et visible touchant l'arrière des dents du haut ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les yeux : les deux paupières complètement fermées, chaque œil devient une ligne courbe douce (cils conservés s'il y en a), comme au milieu d'un clignement ; sourcils, bouche et tout le reste inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les yeux : les deux paupières complètement fermées, chaque œil devient une ligne courbe douce (cils conservés s'il y en a), comme au milieu d'un clignement ; sourcils, bouche et tout le reste inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les yeux : paupières à moitié fermées, la moitié supérieure des yeux couverte, blanc et pupille encore visibles dessous, regard droit ; sourcils, bouche et tout le reste inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les yeux : paupières à moitié fermées, la moitié supérieure des yeux couverte, blanc et pupille encore visibles dessous, regard droit ; sourcils, bouche et tout le reste inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : sourcils légèrement relevés et détendus, yeux un peu plissés par un sourire (paupières inférieures remontées), expression joyeuse ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : sourcils légèrement relevés et détendus, yeux un peu plissés par un sourire (paupières inférieures remontées), expression joyeuse ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : sourcils nettement relevés, yeux plus grands et bien ouverts, expression de surprise ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : sourcils nettement relevés, yeux plus grands et bien ouverts, expression de surprise ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : sourcils abaissés et légèrement froncés vers le centre, regard concentré et déterminé, sans colère ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : sourcils abaissés et légèrement froncés vers le centre, regard concentré et déterminé, sans colère ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : un sourcil légèrement relevé, l'autre au repos, regard tourné vers le haut et le côté comme quelqu'un qui réfléchit ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : un sourcil légèrement relevé, l'autre au repos, regard tourné vers le haut et le côté comme quelqu'un qui réfléchit ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les iris et pupilles des deux yeux sont déplacés vers la gauche de l'image (le personnage regarde vers sa droite, hors caméra) ; paupières, sourcils et bouche exactement comme la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les iris et pupilles des deux yeux sont déplacés vers la gauche de l'image (le personnage regarde vers sa droite, hors caméra) ; paupières, sourcils et bouche exactement comme la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -1229,7 +1229,7 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les iris et pupilles des deux yeux sont déplacés vers la droite de l'image (le personnage regarde vers sa gauche, hors caméra) ; paupières, sourcils et bouche exactement comme la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les iris et pupilles des deux yeux sont déplacés vers la droite de l'image (le personnage regarde vers sa gauche, hors caméra) ; paupières, sourcils et bouche exactement comme la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les iris et pupilles des deux yeux sont déplacés vers le haut, comme quelqu'un qui cherche ses mots ; paupières ouvertes comme la base, sourcils et bouche inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les iris et pupilles des deux yeux sont déplacés vers le haut, comme quelqu'un qui cherche ses mots ; paupières ouvertes comme la base, sourcils et bouche inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : fermée avec un vrai sourire, coins des lèvres nettement relevés ; les yeux et les sourcils ne changent pas (pas de plissement). Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : fermée avec un vrai sourire, coins des lèvres nettement relevés ; les yeux et les sourcils ne changent pas (pas de plissement). Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : grand sourire ouvert montrant les dents du haut serrées contre celles du bas, coins relevés ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : grand sourire ouvert montrant les dents du haut serrées contre celles du bas, coins relevés ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -1349,7 +1349,7 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : grande ouverte comme sur un « A » rieur, mâchoire abaissée, coins relevés, dents du haut visibles ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : grande ouverte comme sur un « A » rieur, mâchoire abaissée, coins relevés, dents du haut visibles ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : le personnage lève sa main droite (à gauche de l'image) à hauteur de l'épaule, paume ouverte vers la caméra, comme pour dire bonjour ; main et avant-bras entièrement dans le cadre, sans cacher le visage ni le cou ; tête, visage, coiffure, épaules et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : le personnage lève sa main droite (à gauche de l'image) à hauteur de l'épaule, paume ouverte vers la caméra, comme pour dire bonjour ; main et avant-bras entièrement dans le cadre, sans cacher le visage ni le cou ; tête, visage, coiffure, épaules et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les deux mains apparaissent en bas de l'image à hauteur de la poitrine, paumes ouvertes vers le haut, coudes bas, comme quelqu'un qui explique calmement ; mains entièrement dans le cadre sous le menton ; tête, visage et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les deux mains apparaissent en bas de l'image à hauteur de la poitrine, paumes ouvertes vers le haut, coudes bas, comme quelqu'un qui explique calmement ; mains entièrement dans le cadre sous le menton ; tête, visage et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : le personnage lève sa main droite (à gauche de l'image) à hauteur de l'épaule, index tendu vers le haut, autres doigts repliés ; main entièrement dans le cadre, sans cacher le visage ; tête, visage et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : le personnage lève sa main droite (à gauche de l'image) à hauteur de l'épaule, index tendu vers le haut, autres doigts repliés ; main entièrement dans le cadre, sans cacher le visage ; tête, visage et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux longs cheveux bruns ondulés, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : le personnage montre un pouce levé de la main droite (à gauche de l'image), main à hauteur de l'épaule, tournée vers la caméra ; main entièrement dans le cadre, sans cacher le visage ; tête, visage et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : le personnage montre un pouce levé de la main droite (à gauche de l'image), main à hauteur de l'épaule, tournée vers la caméra ; main entièrement dans le cadre, sans cacher le visage ; tête, visage et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
@@ -1488,7 +1488,7 @@
     <row r="30" ht="32" customHeight="1">
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>• Les cheveux longs sont l'élément le plus risqué : chaque mèche doit rester exactement au même endroit sur les 26 images. En cas de doute, refaites l'image.</t>
+          <t>• Les cheveux ondulés sont l'élément le plus risqué : chaque mèche doit rester exactement au même endroit sur les 26 images. En cas de doute, refaites l'image.</t>
         </is>
       </c>
     </row>
@@ -1502,15 +1502,23 @@
     <row r="32" ht="32" customHeight="1">
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>• L'original a la bouche ouverte souriante : la base (ligne 0) doit la fermer, c'est la seule modification demandée.</t>
+          <t>• L'original sourit bouche fermée : la base (ligne 0) doit avoir une bouche vraiment neutre, lèvres rouges fermées sans coins relevés (le sourire viendra de bouche_X_sourire et de l'émotion enjoué).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="32" customHeight="1">
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>• Sur toutes les bouches, précisez que le rouge à lèvres reste identique (même teinte, même contour), seule l'ouverture change.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="B30:F30"/>
     <mergeCell ref="B31:F31"/>
     <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B33:F33"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1522,7 +1530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1586,7 +1594,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Voici mon personnage de référence (image jointe). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage (buste centré, tête au même endroit), même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche est fermée, détendue et neutre (pas de sourire, pas de dents visibles), les yeux ouverts (blanc de l'œil et pupille visibles) regardant droit vers la caméra, sourcils au repos, expression calme et neutre. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici mon personnage de référence (image jointe). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage (buste centré, tête au même endroit), même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche est fermée, détendue et neutre (pas de sourire, pas de dents visibles), les yeux ouverts (blanc de l'œil et pupille visibles) regardant droit vers la caméra, sourcils au repos, expression calme et neutre. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
@@ -1646,7 +1654,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres fermées et légèrement pressées l'une contre l'autre, comme au début du son « M » ou « P », un peu plus fermes que dans la base ; yeux, sourcils et tout le reste inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres fermées et légèrement pressées l'une contre l'autre, comme au début du son « M » ou « P », un peu plus fermes que dans la base ; yeux, sourcils et tout le reste inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -1676,7 +1684,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres légèrement entrouvertes laissant voir les dents du haut et du bas serrées, ouverture très faible, pas de langue ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres légèrement entrouvertes laissant voir les dents du haut et du bas serrées, ouverture très faible, pas de langue ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -1706,7 +1714,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : ouverte à moitié, forme légèrement ovale, dents du haut visibles, mâchoire un peu abaissée ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : ouverte à moitié, forme légèrement ovale, dents du haut visibles, mâchoire un peu abaissée ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -1736,7 +1744,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : grande ouverte, mâchoire nettement abaissée, forme ovale verticale, dents du haut visibles, intérieur visible ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : grande ouverte, mâchoire nettement abaissée, forme ovale verticale, dents du haut visibles, intérieur visible ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -1766,7 +1774,7 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres arrondies formant un « O » ouvert de taille moyenne, intérieur sombre visible ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres arrondies formant un « O » ouvert de taille moyenne, intérieur sombre visible ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -1796,7 +1804,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres pincées et projetées vers l'avant en un petit cercle serré, comme pour le son « OU » ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres pincées et projetées vers l'avant en un petit cercle serré, comme pour le son « OU » ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -1826,7 +1834,7 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvre inférieure repliée vers l'intérieur, touchant les dents du haut visibles, lèvre supérieure normale, ouverture faible ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvre inférieure repliée vers l'intérieur, touchant les dents du haut visibles, lèvre supérieure normale, ouverture faible ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -1856,7 +1864,7 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : ouverte moyennement, pointe de la langue relevée et visible touchant l'arrière des dents du haut ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : ouverte moyennement, pointe de la langue relevée et visible touchant l'arrière des dents du haut ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -1886,7 +1894,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les yeux : les deux paupières complètement fermées, chaque œil devient une ligne courbe douce (cils conservés s'il y en a), comme au milieu d'un clignement ; sourcils, bouche et tout le reste inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les yeux : les deux paupières complètement fermées, chaque œil devient une ligne courbe douce (cils conservés s'il y en a), comme au milieu d'un clignement ; sourcils, bouche et tout le reste inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -1916,7 +1924,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les yeux : paupières à moitié fermées, la moitié supérieure des yeux couverte, blanc et pupille encore visibles dessous, regard droit ; sourcils, bouche et tout le reste inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les yeux : paupières à moitié fermées, la moitié supérieure des yeux couverte, blanc et pupille encore visibles dessous, regard droit ; sourcils, bouche et tout le reste inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -1946,7 +1954,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : sourcils légèrement relevés et détendus, yeux un peu plissés par un sourire (paupières inférieures remontées), expression joyeuse ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : sourcils légèrement relevés et détendus, yeux un peu plissés par un sourire (paupières inférieures remontées), expression joyeuse ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -1976,7 +1984,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : sourcils nettement relevés, yeux plus grands et bien ouverts, expression de surprise ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : sourcils nettement relevés, yeux plus grands et bien ouverts, expression de surprise ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -2006,7 +2014,7 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : sourcils abaissés et légèrement froncés vers le centre, regard concentré et déterminé, sans colère ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : sourcils abaissés et légèrement froncés vers le centre, regard concentré et déterminé, sans colère ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -2036,7 +2044,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : un sourcil légèrement relevé, l'autre au repos, regard tourné vers le haut et le côté comme quelqu'un qui réfléchit ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : un sourcil légèrement relevé, l'autre au repos, regard tourné vers le haut et le côté comme quelqu'un qui réfléchit ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -2066,7 +2074,7 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les iris et pupilles des deux yeux sont déplacés vers la gauche de l'image (le personnage regarde vers sa droite, hors caméra) ; paupières, sourcils et bouche exactement comme la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les iris et pupilles des deux yeux sont déplacés vers la gauche de l'image (le personnage regarde vers sa droite, hors caméra) ; paupières, sourcils et bouche exactement comme la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -2096,7 +2104,7 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les iris et pupilles des deux yeux sont déplacés vers la droite de l'image (le personnage regarde vers sa gauche, hors caméra) ; paupières, sourcils et bouche exactement comme la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les iris et pupilles des deux yeux sont déplacés vers la droite de l'image (le personnage regarde vers sa gauche, hors caméra) ; paupières, sourcils et bouche exactement comme la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -2126,7 +2134,7 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les iris et pupilles des deux yeux sont déplacés vers le haut, comme quelqu'un qui cherche ses mots ; paupières ouvertes comme la base, sourcils et bouche inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les iris et pupilles des deux yeux sont déplacés vers le haut, comme quelqu'un qui cherche ses mots ; paupières ouvertes comme la base, sourcils et bouche inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -2156,7 +2164,7 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : fermée avec un vrai sourire, coins des lèvres nettement relevés ; les yeux et les sourcils ne changent pas (pas de plissement). Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : fermée avec un vrai sourire, coins des lèvres nettement relevés ; les yeux et les sourcils ne changent pas (pas de plissement). Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -2186,7 +2194,7 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : grand sourire ouvert montrant les dents du haut serrées contre celles du bas, coins relevés ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : grand sourire ouvert montrant les dents du haut serrées contre celles du bas, coins relevés ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -2216,7 +2224,7 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : grande ouverte comme sur un « A » rieur, mâchoire abaissée, coins relevés, dents du haut visibles ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : grande ouverte comme sur un « A » rieur, mâchoire abaissée, coins relevés, dents du haut visibles ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -2246,7 +2254,7 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : le personnage lève sa main droite (à gauche de l'image) à hauteur de l'épaule, paume ouverte vers la caméra, comme pour dire bonjour ; main et avant-bras entièrement dans le cadre, sans cacher le visage ni le cou ; tête, visage, coiffure, épaules et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : le personnage lève sa main droite (à gauche de l'image) à hauteur de l'épaule, paume ouverte vers la caméra, comme pour dire bonjour ; main et avant-bras entièrement dans le cadre, sans cacher le visage ni le cou ; tête, visage, coiffure, épaules et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
@@ -2276,7 +2284,7 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les deux mains apparaissent en bas de l'image à hauteur de la poitrine, paumes ouvertes vers le haut, coudes bas, comme quelqu'un qui explique calmement ; mains entièrement dans le cadre sous le menton ; tête, visage et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les deux mains apparaissent en bas de l'image à hauteur de la poitrine, paumes ouvertes vers le haut, coudes bas, comme quelqu'un qui explique calmement ; mains entièrement dans le cadre sous le menton ; tête, visage et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -2306,7 +2314,7 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : le personnage lève sa main droite (à gauche de l'image) à hauteur de l'épaule, index tendu vers le haut, autres doigts repliés ; main entièrement dans le cadre, sans cacher le visage ; tête, visage et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : le personnage lève sa main droite (à gauche de l'image) à hauteur de l'épaule, index tendu vers le haut, autres doigts repliés ; main entièrement dans le cadre, sans cacher le visage ; tête, visage et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -2336,7 +2344,7 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : le personnage montre un pouce levé de la main droite (à gauche de l'image), main à hauteur de l'épaule, tournée vers la caméra ; main entièrement dans le cadre, sans cacher le visage ; tête, visage et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : marc_base.png). Génère exactement la même image — même personnage (homme chauve à la barbe courte, veste gris anthracite sur chemise blanche ouverte, bras croisés), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : le personnage montre un pouce levé de la main droite (à gauche de l'image), main à hauteur de l'épaule, tournée vers la caméra ; main entièrement dans le cadre, sans cacher le visage ; tête, visage et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : crâne, barbe, veste, chemise, bras croisés, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
@@ -2362,22 +2370,30 @@
     <row r="31" ht="32" customHeight="1">
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>• La barbe entoure la bouche : sur toutes les bouches, insistez pour que la barbe et la moustache ne changent pas de forme, seule l'ouverture des lèvres change.</t>
+          <t>• L'original sourit légèrement : la base (ligne 0) doit avoir une bouche neutre, fermée, sans coins relevés.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="32" customHeight="1">
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>• Les sourcils de l'original sont légèrement asymétriques (un sourcil relevé) : demandez pour la base des sourcils au repos et symétriques, sinon toutes les images hériteront de cette expression.</t>
+          <t>• La barbe entoure la bouche : sur toutes les bouches, insistez pour que la barbe et la moustache ne changent pas de forme, seule l'ouverture des lèvres change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="32" customHeight="1">
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>• Les rides du front et des yeux font partie du personnage : elles doivent rester identiques sur les images de bouches et de regards ; seules les images d'émotion peuvent les modifier.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="B30:F30"/>
     <mergeCell ref="B31:F31"/>
     <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B33:F33"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Docs : prompts ajustés aux avatars retenus (Lydia cheveux lisses)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142Mr13BCgQRDKKKVw1X1e6
</commit_message>
<xml_diff>
--- a/docs/prompts-lydia-marc-othmane.xlsx
+++ b/docs/prompts-lydia-marc-othmane.xlsx
@@ -719,7 +719,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Voici mon personnage de référence (image jointe). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage (buste centré, tête au même endroit), même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche est fermée, détendue et neutre (pas de sourire, pas de dents visibles), les yeux ouverts (blanc de l'œil et pupille visibles) regardant droit vers la caméra, sourcils au repos, expression calme et neutre. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici mon personnage de référence (image jointe). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage (buste centré, tête au même endroit), même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche est fermée, détendue et neutre (pas de sourire, pas de dents visibles), les yeux ouverts (blanc de l'œil et pupille visibles) regardant droit vers la caméra, sourcils au repos, expression calme et neutre. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres fermées et légèrement pressées l'une contre l'autre, comme au début du son « M » ou « P », un peu plus fermes que dans la base ; yeux, sourcils et tout le reste inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres fermées et légèrement pressées l'une contre l'autre, comme au début du son « M » ou « P », un peu plus fermes que dans la base ; yeux, sourcils et tout le reste inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres légèrement entrouvertes laissant voir les dents du haut et du bas serrées, ouverture très faible, pas de langue ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres légèrement entrouvertes laissant voir les dents du haut et du bas serrées, ouverture très faible, pas de langue ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -839,7 +839,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : ouverte à moitié, forme légèrement ovale, dents du haut visibles, mâchoire un peu abaissée ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : ouverte à moitié, forme légèrement ovale, dents du haut visibles, mâchoire un peu abaissée ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : grande ouverte, mâchoire nettement abaissée, forme ovale verticale, dents du haut visibles, intérieur visible ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : grande ouverte, mâchoire nettement abaissée, forme ovale verticale, dents du haut visibles, intérieur visible ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres arrondies formant un « O » ouvert de taille moyenne, intérieur sombre visible ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres arrondies formant un « O » ouvert de taille moyenne, intérieur sombre visible ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres pincées et projetées vers l'avant en un petit cercle serré, comme pour le son « OU » ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvres pincées et projetées vers l'avant en un petit cercle serré, comme pour le son « OU » ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvre inférieure repliée vers l'intérieur, touchant les dents du haut visibles, lèvre supérieure normale, ouverture faible ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : lèvre inférieure repliée vers l'intérieur, touchant les dents du haut visibles, lèvre supérieure normale, ouverture faible ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : ouverte moyennement, pointe de la langue relevée et visible touchant l'arrière des dents du haut ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : ouverte moyennement, pointe de la langue relevée et visible touchant l'arrière des dents du haut ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les yeux : les deux paupières complètement fermées, chaque œil devient une ligne courbe douce (cils conservés s'il y en a), comme au milieu d'un clignement ; sourcils, bouche et tout le reste inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les yeux : les deux paupières complètement fermées, chaque œil devient une ligne courbe douce (cils conservés s'il y en a), comme au milieu d'un clignement ; sourcils, bouche et tout le reste inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les yeux : paupières à moitié fermées, la moitié supérieure des yeux couverte, blanc et pupille encore visibles dessous, regard droit ; sourcils, bouche et tout le reste inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les yeux : paupières à moitié fermées, la moitié supérieure des yeux couverte, blanc et pupille encore visibles dessous, regard droit ; sourcils, bouche et tout le reste inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : sourcils légèrement relevés et détendus, yeux un peu plissés par un sourire (paupières inférieures remontées), expression joyeuse ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : sourcils légèrement relevés et détendus, yeux un peu plissés par un sourire (paupières inférieures remontées), expression joyeuse ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : sourcils nettement relevés, yeux plus grands et bien ouverts, expression de surprise ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : sourcils nettement relevés, yeux plus grands et bien ouverts, expression de surprise ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -1139,7 +1139,7 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : sourcils abaissés et légèrement froncés vers le centre, regard concentré et déterminé, sans colère ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : sourcils abaissés et légèrement froncés vers le centre, regard concentré et déterminé, sans colère ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : un sourcil légèrement relevé, l'autre au repos, regard tourné vers le haut et le côté comme quelqu'un qui réfléchit ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les sourcils et les yeux : un sourcil légèrement relevé, l'autre au repos, regard tourné vers le haut et le côté comme quelqu'un qui réfléchit ; la bouche reste fermée et neutre comme dans la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les iris et pupilles des deux yeux sont déplacés vers la gauche de l'image (le personnage regarde vers sa droite, hors caméra) ; paupières, sourcils et bouche exactement comme la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les iris et pupilles des deux yeux sont déplacés vers la gauche de l'image (le personnage regarde vers sa droite, hors caméra) ; paupières, sourcils et bouche exactement comme la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -1229,7 +1229,7 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les iris et pupilles des deux yeux sont déplacés vers la droite de l'image (le personnage regarde vers sa gauche, hors caméra) ; paupières, sourcils et bouche exactement comme la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les iris et pupilles des deux yeux sont déplacés vers la droite de l'image (le personnage regarde vers sa gauche, hors caméra) ; paupières, sourcils et bouche exactement comme la base. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les iris et pupilles des deux yeux sont déplacés vers le haut, comme quelqu'un qui cherche ses mots ; paupières ouvertes comme la base, sourcils et bouche inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les iris et pupilles des deux yeux sont déplacés vers le haut, comme quelqu'un qui cherche ses mots ; paupières ouvertes comme la base, sourcils et bouche inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : fermée avec un vrai sourire, coins des lèvres nettement relevés ; les yeux et les sourcils ne changent pas (pas de plissement). Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : fermée avec un vrai sourire, coins des lèvres nettement relevés ; les yeux et les sourcils ne changent pas (pas de plissement). Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : grand sourire ouvert montrant les dents du haut serrées contre celles du bas, coins relevés ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : grand sourire ouvert montrant les dents du haut serrées contre celles du bas, coins relevés ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -1349,7 +1349,7 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : grande ouverte comme sur un « A » rieur, mâchoire abaissée, coins relevés, dents du haut visibles ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : la bouche : grande ouverte comme sur un « A » rieur, mâchoire abaissée, coins relevés, dents du haut visibles ; yeux et sourcils inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : le personnage lève sa main droite (à gauche de l'image) à hauteur de l'épaule, paume ouverte vers la caméra, comme pour dire bonjour ; main et avant-bras entièrement dans le cadre, sans cacher le visage ni le cou ; tête, visage, coiffure, épaules et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : le personnage lève sa main droite (à gauche de l'image) à hauteur de l'épaule, paume ouverte vers la caméra, comme pour dire bonjour ; main et avant-bras entièrement dans le cadre, sans cacher le visage ni le cou ; tête, visage, coiffure, épaules et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les deux mains apparaissent en bas de l'image à hauteur de la poitrine, paumes ouvertes vers le haut, coudes bas, comme quelqu'un qui explique calmement ; mains entièrement dans le cadre sous le menton ; tête, visage et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : les deux mains apparaissent en bas de l'image à hauteur de la poitrine, paumes ouvertes vers le haut, coudes bas, comme quelqu'un qui explique calmement ; mains entièrement dans le cadre sous le menton ; tête, visage et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : le personnage lève sa main droite (à gauche de l'image) à hauteur de l'épaule, index tendu vers le haut, autres doigts repliés ; main entièrement dans le cadre, sans cacher le visage ; tête, visage et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : le personnage lève sa main droite (à gauche de l'image) à hauteur de l'épaule, index tendu vers le haut, autres doigts repliés ; main entièrement dans le cadre, sans cacher le visage ; tête, visage et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et ondulés, lèvres rouges, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : le personnage montre un pouce levé de la main droite (à gauche de l'image), main à hauteur de l'épaule, tournée vers la caméra ; main entièrement dans le cadre, sans cacher le visage ; tête, visage et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, rouge à lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
+          <t>Voici l'image de base de mon personnage (image jointe : lydia_base.png). Génère exactement la même image — même personnage (femme aux cheveux bruns mi-longs et lisses, lèvres rosées, blazer rouge bordeaux sur un haut blanc), même cadrage, même tête, même lumière, même fond uni, même style 3D cartoon — avec une seule différence : le personnage montre un pouce levé de la main droite (à gauche de l'image), main à hauteur de l'épaule, tournée vers la caméra ; main entièrement dans le cadre, sans cacher le visage ; tête, visage et fond inchangés. Tout le reste doit rester strictement identique, pixel pour pixel si possible : cheveux (chaque mèche au même endroit), cils, lèvres, blazer rouge, haut blanc, fond. Image carrée 2048 × 2048, PNG.</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
@@ -1488,7 +1488,7 @@
     <row r="30" ht="32" customHeight="1">
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>• Les cheveux ondulés sont l'élément le plus risqué : chaque mèche doit rester exactement au même endroit sur les 26 images. En cas de doute, refaites l'image.</t>
+          <t>• Les cheveux mi-longs sont l'élément le plus risqué : chaque mèche doit rester exactement au même endroit sur les 26 images. En cas de doute, refaites l'image.</t>
         </is>
       </c>
     </row>
@@ -1502,14 +1502,14 @@
     <row r="32" ht="32" customHeight="1">
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>• L'original sourit bouche fermée : la base (ligne 0) doit avoir une bouche vraiment neutre, lèvres rouges fermées sans coins relevés (le sourire viendra de bouche_X_sourire et de l'émotion enjoué).</t>
+          <t>• L'original sourit bouche fermée : la base (ligne 0) doit avoir une bouche vraiment neutre, fermée, sans coins relevés (le sourire viendra de bouche_X_sourire et de l'émotion enjoué).</t>
         </is>
       </c>
     </row>
     <row r="33" ht="32" customHeight="1">
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>• Sur toutes les bouches, précisez que le rouge à lèvres reste identique (même teinte, même contour), seule l'ouverture change.</t>
+          <t>• Sur toutes les bouches, précisez que la teinte des lèvres reste identique, seule l'ouverture change.</t>
         </is>
       </c>
     </row>

</xml_diff>